<commit_message>
Complete CS13 submission per SUBMISSION.md and RUBRIC.md
Add team info and contribution evidence, group and individual reports,
economic rationale in priority reasons, and repo link in README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BwzdqqKXywtpjcsxgqiN6V
</commit_message>
<xml_diff>
--- a/Nhom6_CS13.xlsx
+++ b/Nhom6_CS13.xlsx
@@ -1153,7 +1153,7 @@
       </c>
       <c r="Q5" s="46" t="inlineStr">
         <is>
-          <t>Giá trị cốt lõi (40 bản/ngày × 15–20 phút). Xếp hạng 2 và chỉ chạy thật SAU khi việc 2 qua cổng, vì bộ đề còn 1 lỗi nghiêm trọng. Tỷ lệ đạt bộ đề đã 96,6% (≥ 95%) nên tự tin 0,8, chưa phải 1 vì chưa thử thật.</t>
+          <t>Giá trị cốt lõi: 40 bản/ngày × 15–20 phút ≈ 10–13 giờ bác sĩ/ngày; là thứ bệnh viện trả 15 triệu/khoa/tháng (12.500 đ/bản). Xếp hạng 2 và chỉ chạy thật SAU khi việc 2 qua cổng, vì bộ đề còn 1 lỗi nghiêm trọng. Tỷ lệ đạt bộ đề đã 96,6% (≥ 95%) nên tự tin 0,8, chưa phải 1 vì chưa thử thật.</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="Q6" s="46" t="inlineStr">
         <is>
-          <t>LÀM TRƯỚC: lỗi nghiêm trọng duy nhất là liều insulin tối → sáng; hồ sơ yêu cầu 0 lỗi nghiêm trọng mới được thử nghiệm. "Một lỗi thuốc lọt đến người bệnh là dừng ngay" (BS. Phương). Bằng chứng chắc (tự tin 1), công sức vừa (so khớp với y lệnh có sẵn).</t>
+          <t>LÀM TRƯỚC: lỗi nghiêm trọng duy nhất là liều insulin tối → sáng; hồ sơ yêu cầu 0 lỗi nghiêm trọng mới được thử nghiệm. "Một lỗi thuốc lọt đến người bệnh là dừng ngay" (BS. Phương). Bằng chứng chắc (tự tin 1), công sức vừa (so khớp với y lệnh có sẵn). Kinh tế: cờ thuốc tin cậy là điều kiện để DS kiểm từ 100% xuống 10% → chi phí 11.668 → 4.918 đ/bản, biên 6,7% → 60,7%.</t>
         </is>
       </c>
     </row>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="Q8" s="46" t="inlineStr">
         <is>
-          <t>Chờ, xem lại ở mốc tháng 6: mô hình miễn phí viết lại dễ hiểu đã tốt (rủi ro bị nuốt 0,7); chưa có cách đo người bệnh làm đúng; nội dung đến tay người bệnh nên phải chờ mảng thuốc ổn định 0 lỗi trước.</t>
+          <t>Chờ, xem lại ở mốc tháng 6: mô hình miễn phí viết lại dễ hiểu đã tốt (rủi ro bị nuốt 0,7); chưa có cách đo người bệnh làm đúng; nội dung đến tay người bệnh nên phải chờ mảng thuốc ổn định 0 lỗi trước. Không tăng doanh thu 15 triệu/khoa; kịch bản xấu hết tiền tháng 9 nên không dàn trải.</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="Q9" s="46" t="inlineStr">
         <is>
-          <t>Chờ: hồ sơ ghi "chưa có bộ đề cho ca chuyển khoa" (sẵn sàng đánh giá = 0) và chỉ phủ một phần nhỏ người bệnh. Xem lại tháng 6, khi đã dựng bộ đề ≥ 40 ca chuyển khoa (Sau này).</t>
+          <t>Chờ: hồ sơ ghi "chưa có bộ đề cho ca chuyển khoa" (sẵn sàng đánh giá = 0) và chỉ phủ một phần nhỏ người bệnh. Xem lại tháng 6, khi đã dựng bộ đề ≥ 40 ca chuyển khoa (Sau này). Dựng bộ đề tốn ~20 giờ chuyên gia/vòng — chưa đáng trước khi có hợp đồng trả phí.</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="Q11" s="46" t="inlineStr">
         <is>
-          <t>Thêm vì điều kiện dừng của đề dựa trên tỷ lệ sửa nhiều &gt; 30% hết tháng 3 thử nghiệm: phải đo được từ ngày đầu. Rẻ, dữ liệu (nháp + bản ký) có sẵn trong hệ thống.</t>
+          <t>Thêm vì "tỷ lệ bản nháp bác sĩ phải sửa nhiều" là biến nguy hiểm nhất trong số liệu kinh tế (dòng 7): quá 30% thì bác sĩ bỏ dùng, mất 15 triệu/khoa/tháng; điều kiện dừng hết tháng 3 thử nghiệm cũng dựa trên nó, nên phải đo từ ngày đầu. Rẻ, dữ liệu (nháp + bản ký) có sẵn trong hệ thống.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename product to "Ra Viện" across submission files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BwzdqqKXywtpjcsxgqiN6V
</commit_message>
<xml_diff>
--- a/Nhom6_CS13.xlsx
+++ b/Nhom6_CS13.xlsx
@@ -630,17 +630,18 @@
     <row r="1" ht="17.25" customHeight="1" s="33">
       <c r="A1" s="34" t="inlineStr">
         <is>
-          <t>CS13 · Lộ trình sản phẩm AI — File thực hành · Đề 3 · RaViện</t>
+          <t>CS13 · Lộ trình sản phẩm AI — File thực hành · Đề 3 · Ra Viện</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="33">
       <c r="A2" s="35" t="inlineStr">
         <is>
-          <t>AI in Action · Track 1 · Khóa 4. FILE LÀM BÀI CỦA NHÓM · Đề 3 · RaViện. Dữ liệu của đề nằm trong file CS13_HoSoTinhHuong.pdf; file CS13_Roadmap_Mau.xlsx là bản mẫu đã điền (một sản phẩm khác) để xem cách điền.</t>
-        </is>
-      </c>
-    </row>
+          <t>AI in Action · Track 1 · Khóa 4. FILE LÀM BÀI CỦA NHÓM · Đề 3 · Ra Viện. Dữ liệu của đề nằm trong file CS13_HoSoTinhHuong.pdf; file CS13_Roadmap_Mau.xlsx là bản mẫu đã điền (một sản phẩm khác) để xem cách điền.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="33">
       <c r="A4" s="32" t="inlineStr">
         <is>
@@ -683,6 +684,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="33">
       <c r="A11" s="32" t="inlineStr">
         <is>
@@ -741,6 +743,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="33">
       <c r="A4" s="38" t="inlineStr">
         <is>
@@ -930,6 +933,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="33">
       <c r="A12" s="41" t="inlineStr">
         <is>
@@ -1002,6 +1006,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="39" customHeight="1" s="33">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -1718,6 +1723,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="26.25" customHeight="1" s="33">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -2011,6 +2017,8 @@
         <v/>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="33">
       <c r="A11" s="41" t="inlineStr">
         <is>
@@ -2157,6 +2165,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="15" customHeight="1" s="33">
       <c r="A22" s="53" t="inlineStr">
         <is>
@@ -2212,6 +2221,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="33">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -2446,6 +2456,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="33">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -2564,7 +2575,7 @@
       </c>
       <c r="B9" s="40" t="inlineStr">
         <is>
-          <t>Phần mềm bệnh án của bệnh viện có ra tính năng tóm tắt ra viện không; tỷ lệ bác sĩ còn dùng RaViện mỗi tuần.</t>
+          <t>Phần mềm bệnh án của bệnh viện có ra tính năng tóm tắt ra viện không; tỷ lệ bác sĩ còn dùng Ra Viện mỗi tuần.</t>
         </is>
       </c>
       <c r="C9" s="40" t="inlineStr">
@@ -2600,6 +2611,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="33">
       <c r="A12" s="53" t="inlineStr">
         <is>
@@ -2664,7 +2676,7 @@
       </c>
       <c r="B4" s="40" t="inlineStr">
         <is>
-          <t>Chưa phát hành RaViện. Tháng 1 sửa lỗi liều insulin bằng đối chiếu thuốc với y lệnh cuối, chạy lại bộ đề 45 hồ sơ đến 0 lỗi nghiêm trọng; rồi thử nghiệm 3 tháng tại 1 khoa nội, bác sĩ ký 100%, dược sĩ kiểm thuốc 100%.</t>
+          <t>Chưa phát hành Ra Viện. Tháng 1 sửa lỗi liều insulin bằng đối chiếu thuốc với y lệnh cuối, chạy lại bộ đề 45 hồ sơ đến 0 lỗi nghiêm trọng; rồi thử nghiệm 3 tháng tại 1 khoa nội, bác sĩ ký 100%, dược sĩ kiểm thuốc 100%.</t>
         </is>
       </c>
       <c r="C4" s="58">
@@ -2791,6 +2803,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="33">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -2961,6 +2974,7 @@
     <row r="2" ht="15" customHeight="1" s="33">
       <c r="A2" s="35" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="33">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -3078,10 +3092,13 @@
         <v/>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="33">
       <c r="A12" s="41" t="n"/>
       <c r="D12" s="60" t="n"/>
     </row>
+    <row r="13"/>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="33">
       <c r="A15" s="61" t="inlineStr">
         <is>
@@ -3199,6 +3216,7 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
     <row r="22" ht="15" customHeight="1" s="33">
       <c r="A22" s="53" t="inlineStr">
         <is>

</xml_diff>